<commit_message>
prepare Phase 3.5B-1 validation
</commit_message>
<xml_diff>
--- a/reports/phase3_5/manual_audit.xlsx
+++ b/reports/phase3_5/manual_audit.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R3cca889a171f4336"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="query_overview" sheetId="2" r:id="Rc54922f78c274948"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="primary_answers" sheetId="3" r:id="R84dfa4e9a1ef4b2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="additional_context" sheetId="4" r:id="R912caffef4bd4464"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rda1683536d8b4024"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="query_overview" sheetId="2" r:id="R2a774e0902fd4d52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="primary_answers" sheetId="3" r:id="R49891b5d38124001"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="additional_context" sheetId="4" r:id="Rd04872b4dc864f22"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -609,7 +609,7 @@
         <x:v>next_step</x:v>
       </x:c>
       <x:c r="B8" s="15" t="str">
-        <x:v>Fill only primary_answers annotation columns, then review the resulting failure distribution before Phase 4 design.</x:v>
+        <x:v>Complete parser_qa.xlsx first; only after Parser QA acceptance fill primary_answers annotation columns. Do not enter Phase 4 from automatic or blank fields.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="72" customHeight="1">
@@ -2518,7 +2518,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b2cf8e144e945ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb16e2190666347a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17226,7 +17226,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R287d6ae6b0984abf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73538d01f0d548d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -49632,7 +49632,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc942abe5238e47bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8aecaa939fbb43ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>